<commit_message>
feat: Add DeepSeek LLM support + major Visualization & Docking improvements
- Integrated DeepSeek as new LLM provider
- Fixed 3D visualization rendering for protein and ligand
- Improved rigid receptor PDBQT preparation
- Enhanced docking workflow stability and error handling
- Better dependency management across modules
</commit_message>
<xml_diff>
--- a/outputs/comparison/tool_comparison.xlsx
+++ b/outputs/comparison/tool_comparison.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison Benchmark" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Comparison Benchmark" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>250</v>
+        <v>615.4</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>14</v>
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>140.8</v>
+        <v>206.7</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>217</v>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>221.3</v>
+        <v>2038.3</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>24</v>

</xml_diff>

<commit_message>
Recover visualization docking DeepSeek integration after security history rewrite
</commit_message>
<xml_diff>
--- a/outputs/comparison/tool_comparison.xlsx
+++ b/outputs/comparison/tool_comparison.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison Benchmark" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Comparison Benchmark" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>250</v>
+        <v>615.4</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>14</v>
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>140.8</v>
+        <v>206.7</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>217</v>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>221.3</v>
+        <v>2038.3</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>24</v>

</xml_diff>

<commit_message>
Recover visualization docking DeepSeek integration
</commit_message>
<xml_diff>
--- a/outputs/comparison/tool_comparison.xlsx
+++ b/outputs/comparison/tool_comparison.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison Benchmark" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Comparison Benchmark" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>250</v>
+        <v>615.4</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>14</v>
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>140.8</v>
+        <v>206.7</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>217</v>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>221.3</v>
+        <v>2038.3</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>24</v>

</xml_diff>